<commit_message>
Work on Admin leave management
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/OrangeHRM_TestData.xlsx
+++ b/src/test/resources/testdata/OrangeHRM_TestData.xlsx
@@ -3,15 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{2D5C80F2-0501-43E0-97CB-AA7DC89561B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9008CA5-228B-41F5-B15D-6023C1183127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4668" yWindow="3708" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Leave Test data" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -59,10 +58,10 @@
     <t>Pending Approval</t>
   </si>
   <si>
-    <t>Ravi M B</t>
-  </si>
-  <si>
     <t>2026-01-01</t>
+  </si>
+  <si>
+    <t>emp 1</t>
   </si>
 </sst>
 </file>
@@ -450,7 +449,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>
@@ -459,7 +458,7 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>